<commit_message>
Add JSON response files for client cases: caso_03_cliente_a_nacional and caso_07_cliente_d_impo_expo
- Added caso_03_cliente_a_nacional.json with details for national client case.
- Added caso_07_cliente_d_impo_expo.json for import/export client case.
</commit_message>
<xml_diff>
--- a/tests/evaluacion-ia/dataset/casos/caso_05_cliente_c_region_1.xlsx
+++ b/tests/evaluacion-ia/dataset/casos/caso_05_cliente_c_region_1.xlsx
@@ -2918,25 +2918,17 @@
         </is>
       </c>
       <c r="D24" s="270" t="n"/>
-      <c r="E24" s="271" t="n">
-        <v>780000</v>
-      </c>
+      <c r="E24" s="271" t="n"/>
       <c r="F24" s="270" t="n"/>
-      <c r="G24" s="271" t="n">
-        <v>1082000</v>
-      </c>
+      <c r="G24" s="271" t="n"/>
       <c r="H24" s="270" t="n"/>
-      <c r="I24" s="271" t="n">
-        <v>1132000</v>
-      </c>
+      <c r="I24" s="271" t="n"/>
       <c r="J24" s="270" t="n"/>
-      <c r="K24" s="271" t="n">
-        <v>1230000</v>
-      </c>
+      <c r="K24" s="271" t="n"/>
       <c r="L24" s="270" t="n"/>
       <c r="M24" s="13" t="n"/>
       <c r="O24" s="56" t="n">
-        <v>1211000</v>
+        <v>821000</v>
       </c>
       <c r="P24" s="50" t="n"/>
     </row>
@@ -2948,25 +2940,17 @@
         </is>
       </c>
       <c r="D25" s="270" t="n"/>
-      <c r="E25" s="271" t="n">
-        <v>1437000</v>
-      </c>
+      <c r="E25" s="271" t="n"/>
       <c r="F25" s="270" t="n"/>
-      <c r="G25" s="271" t="n">
-        <v>1277000</v>
-      </c>
+      <c r="G25" s="271" t="n"/>
       <c r="H25" s="270" t="n"/>
-      <c r="I25" s="271" t="n">
-        <v>2400000</v>
-      </c>
+      <c r="I25" s="271" t="n"/>
       <c r="J25" s="270" t="n"/>
-      <c r="K25" s="271" t="n">
-        <v>1486000</v>
-      </c>
+      <c r="K25" s="271" t="n"/>
       <c r="L25" s="270" t="n"/>
       <c r="M25" s="13" t="n"/>
       <c r="O25" s="57" t="n">
-        <v>2162000</v>
+        <v>1493000</v>
       </c>
     </row>
     <row r="26" ht="20.1" customHeight="1" s="49">
@@ -2977,25 +2961,17 @@
         </is>
       </c>
       <c r="D26" s="270" t="n"/>
-      <c r="E26" s="271" t="n">
-        <v>3704000</v>
-      </c>
+      <c r="E26" s="271" t="n"/>
       <c r="F26" s="270" t="n"/>
-      <c r="G26" s="271" t="n">
-        <v>4310000</v>
-      </c>
+      <c r="G26" s="271" t="n"/>
       <c r="H26" s="270" t="n"/>
-      <c r="I26" s="271" t="n">
-        <v>3604000</v>
-      </c>
+      <c r="I26" s="271" t="n"/>
       <c r="J26" s="270" t="n"/>
-      <c r="K26" s="271" t="n">
-        <v>3636000</v>
-      </c>
+      <c r="K26" s="271" t="n"/>
       <c r="L26" s="270" t="n"/>
       <c r="M26" s="13" t="n"/>
       <c r="O26" s="57" t="n">
-        <v>3151000</v>
+        <v>2850000</v>
       </c>
     </row>
     <row r="27" ht="20.1" customHeight="1" s="49">
@@ -3006,25 +2982,17 @@
         </is>
       </c>
       <c r="D27" s="270" t="n"/>
-      <c r="E27" s="271" t="n">
-        <v>3504000</v>
-      </c>
+      <c r="E27" s="271" t="n"/>
       <c r="F27" s="270" t="n"/>
-      <c r="G27" s="271" t="n">
-        <v>5189000</v>
-      </c>
+      <c r="G27" s="271" t="n"/>
       <c r="H27" s="270" t="n"/>
-      <c r="I27" s="271" t="n">
-        <v>3007000</v>
-      </c>
+      <c r="I27" s="271" t="n"/>
       <c r="J27" s="270" t="n"/>
-      <c r="K27" s="271" t="n">
-        <v>4703000</v>
-      </c>
+      <c r="K27" s="271" t="n"/>
       <c r="L27" s="270" t="n"/>
       <c r="M27" s="13" t="n"/>
       <c r="O27" s="57" t="n">
-        <v>5809000</v>
+        <v>5469000</v>
       </c>
     </row>
     <row r="28" ht="20.1" customHeight="1" s="49">
@@ -3035,25 +3003,17 @@
         </is>
       </c>
       <c r="D28" s="270" t="n"/>
-      <c r="E28" s="271" t="n">
-        <v>3156000</v>
-      </c>
+      <c r="E28" s="271" t="n"/>
       <c r="F28" s="270" t="n"/>
-      <c r="G28" s="271" t="n">
-        <v>4673000</v>
-      </c>
+      <c r="G28" s="271" t="n"/>
       <c r="H28" s="270" t="n"/>
-      <c r="I28" s="271" t="n">
-        <v>2986000</v>
-      </c>
+      <c r="I28" s="271" t="n"/>
       <c r="J28" s="270" t="n"/>
-      <c r="K28" s="271" t="n">
-        <v>5455000</v>
-      </c>
+      <c r="K28" s="271" t="n"/>
       <c r="L28" s="270" t="n"/>
       <c r="M28" s="13" t="n"/>
       <c r="O28" s="58" t="n">
-        <v>3700000</v>
+        <v>5332000</v>
       </c>
     </row>
     <row r="29" ht="5.1" customHeight="1" s="49" thickBot="1">
@@ -3106,25 +3066,17 @@
         </is>
       </c>
       <c r="D32" s="270" t="n"/>
-      <c r="E32" s="271" t="n">
-        <v>1675000</v>
-      </c>
+      <c r="E32" s="271" t="n"/>
       <c r="F32" s="270" t="n"/>
-      <c r="G32" s="271" t="n">
-        <v>1516000</v>
-      </c>
+      <c r="G32" s="271" t="n"/>
       <c r="H32" s="270" t="n"/>
-      <c r="I32" s="271" t="n">
-        <v>1388000</v>
-      </c>
+      <c r="I32" s="271" t="n"/>
       <c r="J32" s="270" t="n"/>
-      <c r="K32" s="271" t="n">
-        <v>1729000</v>
-      </c>
+      <c r="K32" s="271" t="n"/>
       <c r="L32" s="270" t="n"/>
       <c r="M32" s="13" t="n"/>
       <c r="O32" s="56" t="n">
-        <v>1424000</v>
+        <v>1400000</v>
       </c>
     </row>
     <row r="33" ht="20.1" customHeight="1" s="49">
@@ -3135,25 +3087,17 @@
         </is>
       </c>
       <c r="D33" s="270" t="n"/>
-      <c r="E33" s="271" t="n">
-        <v>3075000</v>
-      </c>
+      <c r="E33" s="271" t="n"/>
       <c r="F33" s="270" t="n"/>
-      <c r="G33" s="271" t="n">
-        <v>6138000</v>
-      </c>
+      <c r="G33" s="271" t="n"/>
       <c r="H33" s="270" t="n"/>
-      <c r="I33" s="271" t="n">
-        <v>3250000</v>
-      </c>
+      <c r="I33" s="271" t="n"/>
       <c r="J33" s="270" t="n"/>
-      <c r="K33" s="271" t="n">
-        <v>4232000</v>
-      </c>
+      <c r="K33" s="271" t="n"/>
       <c r="L33" s="270" t="n"/>
       <c r="M33" s="13" t="n"/>
       <c r="O33" s="57" t="n">
-        <v>2778000</v>
+        <v>3592000</v>
       </c>
     </row>
     <row r="34" ht="20.1" customHeight="1" s="49">
@@ -3164,25 +3108,17 @@
         </is>
       </c>
       <c r="D34" s="270" t="n"/>
-      <c r="E34" s="271" t="n">
-        <v>4828000</v>
-      </c>
+      <c r="E34" s="271" t="n"/>
       <c r="F34" s="270" t="n"/>
-      <c r="G34" s="271" t="n">
-        <v>4461000</v>
-      </c>
+      <c r="G34" s="271" t="n"/>
       <c r="H34" s="270" t="n"/>
-      <c r="I34" s="271" t="n">
-        <v>5119000</v>
-      </c>
+      <c r="I34" s="271" t="n"/>
       <c r="J34" s="270" t="n"/>
-      <c r="K34" s="271" t="n">
-        <v>4515000</v>
-      </c>
+      <c r="K34" s="271" t="n"/>
       <c r="L34" s="270" t="n"/>
       <c r="M34" s="13" t="n"/>
       <c r="O34" s="57" t="n">
-        <v>5287000</v>
+        <v>5896000</v>
       </c>
     </row>
     <row r="35" ht="20.1" customHeight="1" s="49">
@@ -3193,25 +3129,17 @@
         </is>
       </c>
       <c r="D35" s="270" t="n"/>
-      <c r="E35" s="271" t="n">
-        <v>4002000</v>
-      </c>
+      <c r="E35" s="271" t="n"/>
       <c r="F35" s="270" t="n"/>
-      <c r="G35" s="271" t="n">
-        <v>5165000</v>
-      </c>
+      <c r="G35" s="271" t="n"/>
       <c r="H35" s="270" t="n"/>
-      <c r="I35" s="271" t="n">
-        <v>5456000</v>
-      </c>
+      <c r="I35" s="271" t="n"/>
       <c r="J35" s="270" t="n"/>
-      <c r="K35" s="271" t="n">
-        <v>4406000</v>
-      </c>
+      <c r="K35" s="271" t="n"/>
       <c r="L35" s="270" t="n"/>
       <c r="M35" s="13" t="n"/>
       <c r="O35" s="57" t="n">
-        <v>5029000</v>
+        <v>4036000</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="49">
@@ -3222,25 +3150,17 @@
         </is>
       </c>
       <c r="D36" s="270" t="n"/>
-      <c r="E36" s="271" t="n">
-        <v>906000</v>
-      </c>
+      <c r="E36" s="271" t="n"/>
       <c r="F36" s="270" t="n"/>
-      <c r="G36" s="271" t="n">
-        <v>764000</v>
-      </c>
+      <c r="G36" s="271" t="n"/>
       <c r="H36" s="270" t="n"/>
-      <c r="I36" s="271" t="n">
-        <v>1853000</v>
-      </c>
+      <c r="I36" s="271" t="n"/>
       <c r="J36" s="270" t="n"/>
-      <c r="K36" s="271" t="n">
-        <v>1095000</v>
-      </c>
+      <c r="K36" s="271" t="n"/>
       <c r="L36" s="270" t="n"/>
       <c r="M36" s="13" t="n"/>
       <c r="O36" s="57" t="n">
-        <v>645000</v>
+        <v>1376000</v>
       </c>
     </row>
     <row r="37" ht="20.1" customHeight="1" s="49">
@@ -3251,25 +3171,17 @@
         </is>
       </c>
       <c r="D37" s="270" t="n"/>
-      <c r="E37" s="271" t="n">
-        <v>1283000</v>
-      </c>
+      <c r="E37" s="271" t="n"/>
       <c r="F37" s="270" t="n"/>
-      <c r="G37" s="271" t="n">
-        <v>739000</v>
-      </c>
+      <c r="G37" s="271" t="n"/>
       <c r="H37" s="270" t="n"/>
-      <c r="I37" s="271" t="n">
-        <v>868000</v>
-      </c>
+      <c r="I37" s="271" t="n"/>
       <c r="J37" s="270" t="n"/>
-      <c r="K37" s="271" t="n">
-        <v>1148000</v>
-      </c>
+      <c r="K37" s="271" t="n"/>
       <c r="L37" s="270" t="n"/>
       <c r="M37" s="13" t="n"/>
       <c r="O37" s="57" t="n">
-        <v>1366000</v>
+        <v>1148000</v>
       </c>
     </row>
     <row r="38" ht="20.1" customHeight="1" s="49">
@@ -3280,25 +3192,17 @@
         </is>
       </c>
       <c r="D38" s="270" t="n"/>
-      <c r="E38" s="271" t="n">
-        <v>883000</v>
-      </c>
+      <c r="E38" s="271" t="n"/>
       <c r="F38" s="270" t="n"/>
-      <c r="G38" s="271" t="n">
-        <v>1124000</v>
-      </c>
+      <c r="G38" s="271" t="n"/>
       <c r="H38" s="270" t="n"/>
-      <c r="I38" s="271" t="n">
-        <v>909000</v>
-      </c>
+      <c r="I38" s="271" t="n"/>
       <c r="J38" s="270" t="n"/>
-      <c r="K38" s="271" t="n">
-        <v>1239000</v>
-      </c>
+      <c r="K38" s="271" t="n"/>
       <c r="L38" s="270" t="n"/>
       <c r="M38" s="13" t="n"/>
       <c r="O38" s="58" t="n">
-        <v>1350000</v>
+        <v>1377000</v>
       </c>
     </row>
     <row r="39" ht="5.1" customHeight="1" s="49" thickBot="1">
@@ -3351,25 +3255,17 @@
         </is>
       </c>
       <c r="D42" s="270" t="n"/>
-      <c r="E42" s="271" t="n">
-        <v>4242000</v>
-      </c>
+      <c r="E42" s="271" t="n"/>
       <c r="F42" s="270" t="n"/>
-      <c r="G42" s="271" t="n">
-        <v>3648000</v>
-      </c>
+      <c r="G42" s="271" t="n"/>
       <c r="H42" s="270" t="n"/>
-      <c r="I42" s="271" t="n">
-        <v>2841000</v>
-      </c>
+      <c r="I42" s="271" t="n"/>
       <c r="J42" s="270" t="n"/>
-      <c r="K42" s="271" t="n">
-        <v>2891000</v>
-      </c>
+      <c r="K42" s="271" t="n"/>
       <c r="L42" s="270" t="n"/>
       <c r="M42" s="13" t="n"/>
       <c r="O42" s="56" t="n">
-        <v>2819000</v>
+        <v>3545000</v>
       </c>
     </row>
     <row r="43" ht="20.1" customHeight="1" s="49">
@@ -3380,25 +3276,17 @@
         </is>
       </c>
       <c r="D43" s="270" t="n"/>
-      <c r="E43" s="271" t="n">
-        <v>3959000</v>
-      </c>
+      <c r="E43" s="271" t="n"/>
       <c r="F43" s="270" t="n"/>
-      <c r="G43" s="271" t="n">
-        <v>2963000</v>
-      </c>
+      <c r="G43" s="271" t="n"/>
       <c r="H43" s="270" t="n"/>
-      <c r="I43" s="271" t="n">
-        <v>2860000</v>
-      </c>
+      <c r="I43" s="271" t="n"/>
       <c r="J43" s="270" t="n"/>
-      <c r="K43" s="271" t="n">
-        <v>3996000</v>
-      </c>
+      <c r="K43" s="271" t="n"/>
       <c r="L43" s="270" t="n"/>
       <c r="M43" s="13" t="n"/>
       <c r="O43" s="57" t="n">
-        <v>2833000</v>
+        <v>3967000</v>
       </c>
     </row>
     <row r="44" ht="20.1" customHeight="1" s="49">
@@ -3409,25 +3297,17 @@
         </is>
       </c>
       <c r="D44" s="270" t="n"/>
-      <c r="E44" s="271" t="n">
-        <v>4550000</v>
-      </c>
+      <c r="E44" s="271" t="n"/>
       <c r="F44" s="270" t="n"/>
-      <c r="G44" s="271" t="n">
-        <v>5409000</v>
-      </c>
+      <c r="G44" s="271" t="n"/>
       <c r="H44" s="270" t="n"/>
-      <c r="I44" s="271" t="n">
-        <v>3161000</v>
-      </c>
+      <c r="I44" s="271" t="n"/>
       <c r="J44" s="270" t="n"/>
-      <c r="K44" s="271" t="n">
-        <v>2773000</v>
-      </c>
+      <c r="K44" s="271" t="n"/>
       <c r="L44" s="270" t="n"/>
       <c r="M44" s="13" t="n"/>
       <c r="O44" s="57" t="n">
-        <v>3725000</v>
+        <v>4258000</v>
       </c>
     </row>
     <row r="45" ht="20.1" customHeight="1" s="49">
@@ -3438,25 +3318,17 @@
         </is>
       </c>
       <c r="D45" s="270" t="n"/>
-      <c r="E45" s="271" t="n">
-        <v>4191000</v>
-      </c>
+      <c r="E45" s="271" t="n"/>
       <c r="F45" s="270" t="n"/>
-      <c r="G45" s="271" t="n">
-        <v>4002000</v>
-      </c>
+      <c r="G45" s="271" t="n"/>
       <c r="H45" s="270" t="n"/>
-      <c r="I45" s="271" t="n">
-        <v>5670000</v>
-      </c>
+      <c r="I45" s="271" t="n"/>
       <c r="J45" s="270" t="n"/>
-      <c r="K45" s="271" t="n">
-        <v>4637000</v>
-      </c>
+      <c r="K45" s="271" t="n"/>
       <c r="L45" s="270" t="n"/>
       <c r="M45" s="13" t="n"/>
       <c r="O45" s="57" t="n">
-        <v>6365000</v>
+        <v>3637000</v>
       </c>
     </row>
     <row r="46" ht="20.1" customHeight="1" s="49">
@@ -3467,25 +3339,17 @@
         </is>
       </c>
       <c r="D46" s="270" t="n"/>
-      <c r="E46" s="271" t="n">
-        <v>1112000</v>
-      </c>
+      <c r="E46" s="271" t="n"/>
       <c r="F46" s="270" t="n"/>
-      <c r="G46" s="271" t="n">
-        <v>1475000</v>
-      </c>
+      <c r="G46" s="271" t="n"/>
       <c r="H46" s="270" t="n"/>
-      <c r="I46" s="271" t="n">
-        <v>1550000</v>
-      </c>
+      <c r="I46" s="271" t="n"/>
       <c r="J46" s="270" t="n"/>
-      <c r="K46" s="271" t="n">
-        <v>2931000</v>
-      </c>
+      <c r="K46" s="271" t="n"/>
       <c r="L46" s="270" t="n"/>
       <c r="M46" s="13" t="n"/>
       <c r="O46" s="57" t="n">
-        <v>1270000</v>
+        <v>1963000</v>
       </c>
     </row>
     <row r="47" ht="20.1" customHeight="1" s="49">
@@ -3496,25 +3360,17 @@
         </is>
       </c>
       <c r="D47" s="270" t="n"/>
-      <c r="E47" s="271" t="n">
-        <v>961000</v>
-      </c>
+      <c r="E47" s="271" t="n"/>
       <c r="F47" s="270" t="n"/>
-      <c r="G47" s="271" t="n">
-        <v>1485000</v>
-      </c>
+      <c r="G47" s="271" t="n"/>
       <c r="H47" s="270" t="n"/>
-      <c r="I47" s="271" t="n">
-        <v>892000</v>
-      </c>
+      <c r="I47" s="271" t="n"/>
       <c r="J47" s="270" t="n"/>
-      <c r="K47" s="271" t="n">
-        <v>884000</v>
-      </c>
+      <c r="K47" s="271" t="n"/>
       <c r="L47" s="270" t="n"/>
       <c r="M47" s="13" t="n"/>
       <c r="O47" s="58" t="n">
-        <v>1418000</v>
+        <v>666000</v>
       </c>
     </row>
     <row r="48" ht="5.1" customHeight="1" s="49" thickBot="1">
@@ -3568,25 +3424,17 @@
         </is>
       </c>
       <c r="D51" s="270" t="n"/>
-      <c r="E51" s="271" t="n">
-        <v>1564000</v>
-      </c>
+      <c r="E51" s="271" t="n"/>
       <c r="F51" s="270" t="n"/>
-      <c r="G51" s="271" t="n">
-        <v>1591000</v>
-      </c>
+      <c r="G51" s="271" t="n"/>
       <c r="H51" s="270" t="n"/>
-      <c r="I51" s="271" t="n">
-        <v>1440000</v>
-      </c>
+      <c r="I51" s="271" t="n"/>
       <c r="J51" s="270" t="n"/>
-      <c r="K51" s="271" t="n">
-        <v>1060000</v>
-      </c>
+      <c r="K51" s="271" t="n"/>
       <c r="L51" s="270" t="n"/>
       <c r="M51" s="13" t="n"/>
       <c r="O51" s="56" t="n">
-        <v>2050000</v>
+        <v>1899000</v>
       </c>
     </row>
     <row r="52" ht="20.1" customHeight="1" s="49">
@@ -3597,25 +3445,17 @@
         </is>
       </c>
       <c r="D52" s="270" t="n"/>
-      <c r="E52" s="271" t="n">
-        <v>3286000</v>
-      </c>
+      <c r="E52" s="271" t="n"/>
       <c r="F52" s="270" t="n"/>
-      <c r="G52" s="271" t="n">
-        <v>3265000</v>
-      </c>
+      <c r="G52" s="271" t="n"/>
       <c r="H52" s="270" t="n"/>
-      <c r="I52" s="271" t="n">
-        <v>5315000</v>
-      </c>
+      <c r="I52" s="271" t="n"/>
       <c r="J52" s="270" t="n"/>
-      <c r="K52" s="271" t="n">
-        <v>4002000</v>
-      </c>
+      <c r="K52" s="271" t="n"/>
       <c r="L52" s="270" t="n"/>
       <c r="M52" s="13" t="n"/>
       <c r="O52" s="57" t="n">
-        <v>3003000</v>
+        <v>5511000</v>
       </c>
     </row>
     <row r="53" ht="20.1" customHeight="1" s="49">
@@ -3626,25 +3466,17 @@
         </is>
       </c>
       <c r="D53" s="270" t="n"/>
-      <c r="E53" s="271" t="n">
-        <v>3796000</v>
-      </c>
+      <c r="E53" s="271" t="n"/>
       <c r="F53" s="270" t="n"/>
-      <c r="G53" s="271" t="n">
-        <v>5668000</v>
-      </c>
+      <c r="G53" s="271" t="n"/>
       <c r="H53" s="270" t="n"/>
-      <c r="I53" s="271" t="n">
-        <v>4794000</v>
-      </c>
+      <c r="I53" s="271" t="n"/>
       <c r="J53" s="270" t="n"/>
-      <c r="K53" s="271" t="n">
-        <v>3185000</v>
-      </c>
+      <c r="K53" s="271" t="n"/>
       <c r="L53" s="270" t="n"/>
       <c r="M53" s="13" t="n"/>
       <c r="O53" s="57" t="n">
-        <v>3557000</v>
+        <v>3033000</v>
       </c>
     </row>
     <row r="54" ht="20.1" customHeight="1" s="49">
@@ -3655,25 +3487,17 @@
         </is>
       </c>
       <c r="D54" s="270" t="n"/>
-      <c r="E54" s="271" t="n">
-        <v>5346000</v>
-      </c>
+      <c r="E54" s="271" t="n"/>
       <c r="F54" s="270" t="n"/>
-      <c r="G54" s="271" t="n">
-        <v>4178000</v>
-      </c>
+      <c r="G54" s="271" t="n"/>
       <c r="H54" s="270" t="n"/>
-      <c r="I54" s="271" t="n">
-        <v>4581000</v>
-      </c>
+      <c r="I54" s="271" t="n"/>
       <c r="J54" s="270" t="n"/>
-      <c r="K54" s="271" t="n">
-        <v>4477000</v>
-      </c>
+      <c r="K54" s="271" t="n"/>
       <c r="L54" s="270" t="n"/>
       <c r="M54" s="13" t="n"/>
       <c r="O54" s="57" t="n">
-        <v>3819000</v>
+        <v>4230000</v>
       </c>
     </row>
     <row r="55" ht="20.1" customHeight="1" s="49">
@@ -3684,25 +3508,17 @@
         </is>
       </c>
       <c r="D55" s="270" t="n"/>
-      <c r="E55" s="271" t="n">
-        <v>1077000</v>
-      </c>
+      <c r="E55" s="271" t="n"/>
       <c r="F55" s="270" t="n"/>
-      <c r="G55" s="271" t="n">
-        <v>1414000</v>
-      </c>
+      <c r="G55" s="271" t="n"/>
       <c r="H55" s="270" t="n"/>
-      <c r="I55" s="271" t="n">
-        <v>1767000</v>
-      </c>
+      <c r="I55" s="271" t="n"/>
       <c r="J55" s="270" t="n"/>
-      <c r="K55" s="271" t="n">
-        <v>647000</v>
-      </c>
+      <c r="K55" s="271" t="n"/>
       <c r="L55" s="270" t="n"/>
       <c r="M55" s="13" t="n"/>
       <c r="O55" s="57" t="n">
-        <v>813000</v>
+        <v>661000</v>
       </c>
     </row>
     <row r="56" ht="20.1" customHeight="1" s="49">
@@ -3713,25 +3529,17 @@
         </is>
       </c>
       <c r="D56" s="270" t="n"/>
-      <c r="E56" s="271" t="n">
-        <v>1170000</v>
-      </c>
+      <c r="E56" s="271" t="n"/>
       <c r="F56" s="270" t="n"/>
-      <c r="G56" s="271" t="n">
-        <v>972000</v>
-      </c>
+      <c r="G56" s="271" t="n"/>
       <c r="H56" s="270" t="n"/>
-      <c r="I56" s="271" t="n">
-        <v>1815000</v>
-      </c>
+      <c r="I56" s="271" t="n"/>
       <c r="J56" s="270" t="n"/>
-      <c r="K56" s="271" t="n">
-        <v>749000</v>
-      </c>
+      <c r="K56" s="271" t="n"/>
       <c r="L56" s="270" t="n"/>
       <c r="M56" s="13" t="n"/>
       <c r="O56" s="57" t="n">
-        <v>1364000</v>
+        <v>1353000</v>
       </c>
     </row>
     <row r="57" ht="20.1" customHeight="1" s="49">
@@ -3742,25 +3550,17 @@
         </is>
       </c>
       <c r="D57" s="270" t="n"/>
-      <c r="E57" s="271" t="n">
-        <v>1020000</v>
-      </c>
+      <c r="E57" s="271" t="n"/>
       <c r="F57" s="270" t="n"/>
-      <c r="G57" s="271" t="n">
-        <v>1451000</v>
-      </c>
+      <c r="G57" s="271" t="n"/>
       <c r="H57" s="270" t="n"/>
-      <c r="I57" s="271" t="n">
-        <v>840000</v>
-      </c>
+      <c r="I57" s="271" t="n"/>
       <c r="J57" s="270" t="n"/>
-      <c r="K57" s="271" t="n">
-        <v>1289000</v>
-      </c>
+      <c r="K57" s="271" t="n"/>
       <c r="L57" s="270" t="n"/>
       <c r="M57" s="13" t="n"/>
       <c r="O57" s="58" t="n">
-        <v>1463000</v>
+        <v>842000</v>
       </c>
     </row>
     <row r="58" ht="5.1" customHeight="1" s="49" thickBot="1">
@@ -3813,25 +3613,17 @@
         </is>
       </c>
       <c r="D61" s="270" t="n"/>
-      <c r="E61" s="271" t="n">
-        <v>2837000</v>
-      </c>
+      <c r="E61" s="271" t="n"/>
       <c r="F61" s="270" t="n"/>
-      <c r="G61" s="271" t="n">
-        <v>2369000</v>
-      </c>
+      <c r="G61" s="271" t="n"/>
       <c r="H61" s="270" t="n"/>
-      <c r="I61" s="271" t="n">
-        <v>2148000</v>
-      </c>
+      <c r="I61" s="271" t="n"/>
       <c r="J61" s="270" t="n"/>
-      <c r="K61" s="271" t="n">
-        <v>3811000</v>
-      </c>
+      <c r="K61" s="271" t="n"/>
       <c r="L61" s="270" t="n"/>
       <c r="M61" s="13" t="n"/>
       <c r="O61" s="56" t="n">
-        <v>3843000</v>
+        <v>3101000</v>
       </c>
     </row>
     <row r="62" ht="20.1" customHeight="1" s="49">
@@ -3842,25 +3634,17 @@
         </is>
       </c>
       <c r="D62" s="270" t="n"/>
-      <c r="E62" s="271" t="n">
-        <v>4729000</v>
-      </c>
+      <c r="E62" s="271" t="n"/>
       <c r="F62" s="270" t="n"/>
-      <c r="G62" s="271" t="n">
-        <v>4479000</v>
-      </c>
+      <c r="G62" s="271" t="n"/>
       <c r="H62" s="270" t="n"/>
-      <c r="I62" s="271" t="n">
-        <v>2992000</v>
-      </c>
+      <c r="I62" s="271" t="n"/>
       <c r="J62" s="270" t="n"/>
-      <c r="K62" s="271" t="n">
-        <v>2871000</v>
-      </c>
+      <c r="K62" s="271" t="n"/>
       <c r="L62" s="270" t="n"/>
       <c r="M62" s="13" t="n"/>
       <c r="O62" s="57" t="n">
-        <v>2083000</v>
+        <v>3308000</v>
       </c>
     </row>
     <row r="63" ht="20.1" customHeight="1" s="49">
@@ -3871,25 +3655,17 @@
         </is>
       </c>
       <c r="D63" s="270" t="n"/>
-      <c r="E63" s="271" t="n">
-        <v>4901000</v>
-      </c>
+      <c r="E63" s="271" t="n"/>
       <c r="F63" s="270" t="n"/>
-      <c r="G63" s="271" t="n">
-        <v>5926000</v>
-      </c>
+      <c r="G63" s="271" t="n"/>
       <c r="H63" s="270" t="n"/>
-      <c r="I63" s="271" t="n">
-        <v>5463000</v>
-      </c>
+      <c r="I63" s="271" t="n"/>
       <c r="J63" s="270" t="n"/>
-      <c r="K63" s="271" t="n">
-        <v>5166000</v>
-      </c>
+      <c r="K63" s="271" t="n"/>
       <c r="L63" s="270" t="n"/>
       <c r="M63" s="13" t="n"/>
       <c r="O63" s="57" t="n">
-        <v>3087000</v>
+        <v>3410000</v>
       </c>
     </row>
     <row r="64" ht="20.1" customHeight="1" s="49">
@@ -3900,25 +3676,17 @@
         </is>
       </c>
       <c r="D64" s="270" t="n"/>
-      <c r="E64" s="271" t="n">
-        <v>3220000</v>
-      </c>
+      <c r="E64" s="271" t="n"/>
       <c r="F64" s="270" t="n"/>
-      <c r="G64" s="271" t="n">
-        <v>6597000</v>
-      </c>
+      <c r="G64" s="271" t="n"/>
       <c r="H64" s="270" t="n"/>
-      <c r="I64" s="271" t="n">
-        <v>6452000</v>
-      </c>
+      <c r="I64" s="271" t="n"/>
       <c r="J64" s="270" t="n"/>
-      <c r="K64" s="271" t="n">
-        <v>4141000</v>
-      </c>
+      <c r="K64" s="271" t="n"/>
       <c r="L64" s="270" t="n"/>
       <c r="M64" s="13" t="n"/>
       <c r="O64" s="57" t="n">
-        <v>3156000</v>
+        <v>4646000</v>
       </c>
     </row>
     <row r="65" ht="20.1" customHeight="1" s="49">
@@ -3929,25 +3697,17 @@
         </is>
       </c>
       <c r="D65" s="270" t="n"/>
-      <c r="E65" s="271" t="n">
-        <v>1136000</v>
-      </c>
+      <c r="E65" s="271" t="n"/>
       <c r="F65" s="270" t="n"/>
-      <c r="G65" s="271" t="n">
-        <v>1490000</v>
-      </c>
+      <c r="G65" s="271" t="n"/>
       <c r="H65" s="270" t="n"/>
-      <c r="I65" s="271" t="n">
-        <v>907000</v>
-      </c>
+      <c r="I65" s="271" t="n"/>
       <c r="J65" s="270" t="n"/>
-      <c r="K65" s="271" t="n">
-        <v>2964000</v>
-      </c>
+      <c r="K65" s="271" t="n"/>
       <c r="L65" s="270" t="n"/>
       <c r="M65" s="13" t="n"/>
       <c r="O65" s="57" t="n">
-        <v>1580000</v>
+        <v>1595000</v>
       </c>
     </row>
     <row r="66" ht="20.1" customHeight="1" s="49">
@@ -3958,25 +3718,17 @@
         </is>
       </c>
       <c r="D66" s="270" t="n"/>
-      <c r="E66" s="271" t="n">
-        <v>970000</v>
-      </c>
+      <c r="E66" s="271" t="n"/>
       <c r="F66" s="270" t="n"/>
-      <c r="G66" s="271" t="n">
-        <v>889000</v>
-      </c>
+      <c r="G66" s="271" t="n"/>
       <c r="H66" s="270" t="n"/>
-      <c r="I66" s="271" t="n">
-        <v>1808000</v>
-      </c>
+      <c r="I66" s="271" t="n"/>
       <c r="J66" s="270" t="n"/>
-      <c r="K66" s="271" t="n">
-        <v>1206000</v>
-      </c>
+      <c r="K66" s="271" t="n"/>
       <c r="L66" s="270" t="n"/>
       <c r="M66" s="13" t="n"/>
       <c r="O66" s="58" t="n">
-        <v>1133000</v>
+        <v>772000</v>
       </c>
     </row>
     <row r="67" ht="5.1" customHeight="1" s="49" thickBot="1">
@@ -4030,25 +3782,17 @@
         </is>
       </c>
       <c r="D70" s="270" t="n"/>
-      <c r="E70" s="271" t="n">
-        <v>1906000</v>
-      </c>
+      <c r="E70" s="271" t="n"/>
       <c r="F70" s="270" t="n"/>
-      <c r="G70" s="271" t="n">
-        <v>2091000</v>
-      </c>
+      <c r="G70" s="271" t="n"/>
       <c r="H70" s="270" t="n"/>
-      <c r="I70" s="271" t="n">
-        <v>1124000</v>
-      </c>
+      <c r="I70" s="271" t="n"/>
       <c r="J70" s="270" t="n"/>
-      <c r="K70" s="271" t="n">
-        <v>1911000</v>
-      </c>
+      <c r="K70" s="271" t="n"/>
       <c r="L70" s="270" t="n"/>
       <c r="M70" s="13" t="n"/>
       <c r="O70" s="56" t="n">
-        <v>1580000</v>
+        <v>2259000</v>
       </c>
     </row>
     <row r="71" ht="20.1" customHeight="1" s="49">
@@ -4059,25 +3803,17 @@
         </is>
       </c>
       <c r="D71" s="270" t="n"/>
-      <c r="E71" s="271" t="n">
-        <v>4596000</v>
-      </c>
+      <c r="E71" s="271" t="n"/>
       <c r="F71" s="270" t="n"/>
-      <c r="G71" s="271" t="n">
-        <v>5095000</v>
-      </c>
+      <c r="G71" s="271" t="n"/>
       <c r="H71" s="270" t="n"/>
-      <c r="I71" s="271" t="n">
-        <v>4440000</v>
-      </c>
+      <c r="I71" s="271" t="n"/>
       <c r="J71" s="270" t="n"/>
-      <c r="K71" s="271" t="n">
-        <v>3050000</v>
-      </c>
+      <c r="K71" s="271" t="n"/>
       <c r="L71" s="270" t="n"/>
       <c r="M71" s="13" t="n"/>
       <c r="O71" s="57" t="n">
-        <v>4767000</v>
+        <v>3265000</v>
       </c>
     </row>
     <row r="72" ht="20.1" customHeight="1" s="49">
@@ -4088,25 +3824,17 @@
         </is>
       </c>
       <c r="D72" s="270" t="n"/>
-      <c r="E72" s="271" t="n">
-        <v>5293000</v>
-      </c>
+      <c r="E72" s="271" t="n"/>
       <c r="F72" s="270" t="n"/>
-      <c r="G72" s="271" t="n">
-        <v>3128000</v>
-      </c>
+      <c r="G72" s="271" t="n"/>
       <c r="H72" s="270" t="n"/>
-      <c r="I72" s="271" t="n">
-        <v>3437000</v>
-      </c>
+      <c r="I72" s="271" t="n"/>
       <c r="J72" s="270" t="n"/>
-      <c r="K72" s="271" t="n">
-        <v>4828000</v>
-      </c>
+      <c r="K72" s="271" t="n"/>
       <c r="L72" s="270" t="n"/>
       <c r="M72" s="13" t="n"/>
       <c r="O72" s="57" t="n">
-        <v>5379000</v>
+        <v>4678000</v>
       </c>
     </row>
     <row r="73" ht="20.1" customHeight="1" s="49">
@@ -4117,25 +3845,17 @@
         </is>
       </c>
       <c r="D73" s="270" t="n"/>
-      <c r="E73" s="271" t="n">
-        <v>4116000</v>
-      </c>
+      <c r="E73" s="271" t="n"/>
       <c r="F73" s="270" t="n"/>
-      <c r="G73" s="271" t="n">
-        <v>4677000</v>
-      </c>
+      <c r="G73" s="271" t="n"/>
       <c r="H73" s="270" t="n"/>
-      <c r="I73" s="271" t="n">
-        <v>3854000</v>
-      </c>
+      <c r="I73" s="271" t="n"/>
       <c r="J73" s="270" t="n"/>
-      <c r="K73" s="271" t="n">
-        <v>5431000</v>
-      </c>
+      <c r="K73" s="271" t="n"/>
       <c r="L73" s="270" t="n"/>
       <c r="M73" s="13" t="n"/>
       <c r="O73" s="57" t="n">
-        <v>5920000</v>
+        <v>3040000</v>
       </c>
     </row>
     <row r="74" ht="20.1" customHeight="1" s="49">
@@ -4146,25 +3866,17 @@
         </is>
       </c>
       <c r="D74" s="270" t="n"/>
-      <c r="E74" s="271" t="n">
-        <v>731000</v>
-      </c>
+      <c r="E74" s="271" t="n"/>
       <c r="F74" s="270" t="n"/>
-      <c r="G74" s="271" t="n">
-        <v>1089000</v>
-      </c>
+      <c r="G74" s="271" t="n"/>
       <c r="H74" s="270" t="n"/>
-      <c r="I74" s="271" t="n">
-        <v>1239000</v>
-      </c>
+      <c r="I74" s="271" t="n"/>
       <c r="J74" s="270" t="n"/>
-      <c r="K74" s="271" t="n">
-        <v>1354000</v>
-      </c>
+      <c r="K74" s="271" t="n"/>
       <c r="L74" s="270" t="n"/>
       <c r="M74" s="13" t="n"/>
       <c r="O74" s="57" t="n">
-        <v>1286000</v>
+        <v>1156000</v>
       </c>
     </row>
     <row r="75" ht="20.1" customHeight="1" s="49">
@@ -4175,25 +3887,17 @@
         </is>
       </c>
       <c r="D75" s="270" t="n"/>
-      <c r="E75" s="271" t="n">
-        <v>1336000</v>
-      </c>
+      <c r="E75" s="271" t="n"/>
       <c r="F75" s="270" t="n"/>
-      <c r="G75" s="271" t="n">
-        <v>1266000</v>
-      </c>
+      <c r="G75" s="271" t="n"/>
       <c r="H75" s="270" t="n"/>
-      <c r="I75" s="271" t="n">
-        <v>853000</v>
-      </c>
+      <c r="I75" s="271" t="n"/>
       <c r="J75" s="270" t="n"/>
-      <c r="K75" s="271" t="n">
-        <v>664000</v>
-      </c>
+      <c r="K75" s="271" t="n"/>
       <c r="L75" s="270" t="n"/>
       <c r="M75" s="13" t="n"/>
       <c r="O75" s="57" t="n">
-        <v>1007000</v>
+        <v>960000</v>
       </c>
     </row>
     <row r="76" ht="20.1" customHeight="1" s="49">
@@ -4204,25 +3908,17 @@
         </is>
       </c>
       <c r="D76" s="270" t="n"/>
-      <c r="E76" s="271" t="n">
-        <v>1388000</v>
-      </c>
+      <c r="E76" s="271" t="n"/>
       <c r="F76" s="270" t="n"/>
-      <c r="G76" s="271" t="n">
-        <v>1168000</v>
-      </c>
+      <c r="G76" s="271" t="n"/>
       <c r="H76" s="270" t="n"/>
-      <c r="I76" s="271" t="n">
-        <v>862000</v>
-      </c>
+      <c r="I76" s="271" t="n"/>
       <c r="J76" s="270" t="n"/>
-      <c r="K76" s="271" t="n">
-        <v>678000</v>
-      </c>
+      <c r="K76" s="271" t="n"/>
       <c r="L76" s="270" t="n"/>
       <c r="M76" s="13" t="n"/>
       <c r="O76" s="58" t="n">
-        <v>870000</v>
+        <v>1148000</v>
       </c>
     </row>
     <row r="77" ht="5.1" customHeight="1" s="49" thickBot="1">
@@ -4275,25 +3971,17 @@
         </is>
       </c>
       <c r="D80" s="270" t="n"/>
-      <c r="E80" s="271" t="n">
-        <v>3247000</v>
-      </c>
+      <c r="E80" s="271" t="n"/>
       <c r="F80" s="270" t="n"/>
-      <c r="G80" s="271" t="n">
-        <v>4034000</v>
-      </c>
+      <c r="G80" s="271" t="n"/>
       <c r="H80" s="270" t="n"/>
-      <c r="I80" s="271" t="n">
-        <v>3999000</v>
-      </c>
+      <c r="I80" s="271" t="n"/>
       <c r="J80" s="270" t="n"/>
-      <c r="K80" s="271" t="n">
-        <v>3509000</v>
-      </c>
+      <c r="K80" s="271" t="n"/>
       <c r="L80" s="270" t="n"/>
       <c r="M80" s="13" t="n"/>
       <c r="O80" s="56" t="n">
-        <v>3665000</v>
+        <v>3553000</v>
       </c>
     </row>
     <row r="81" ht="20.1" customHeight="1" s="49">
@@ -4304,25 +3992,17 @@
         </is>
       </c>
       <c r="D81" s="270" t="n"/>
-      <c r="E81" s="271" t="n">
-        <v>2496000</v>
-      </c>
+      <c r="E81" s="271" t="n"/>
       <c r="F81" s="270" t="n"/>
-      <c r="G81" s="271" t="n">
-        <v>3066000</v>
-      </c>
+      <c r="G81" s="271" t="n"/>
       <c r="H81" s="270" t="n"/>
-      <c r="I81" s="271" t="n">
-        <v>3425000</v>
-      </c>
+      <c r="I81" s="271" t="n"/>
       <c r="J81" s="270" t="n"/>
-      <c r="K81" s="271" t="n">
-        <v>3803000</v>
-      </c>
+      <c r="K81" s="271" t="n"/>
       <c r="L81" s="270" t="n"/>
       <c r="M81" s="13" t="n"/>
       <c r="O81" s="57" t="n">
-        <v>4069000</v>
+        <v>3914000</v>
       </c>
     </row>
     <row r="82" ht="20.1" customHeight="1" s="49">
@@ -4333,25 +4013,17 @@
         </is>
       </c>
       <c r="D82" s="270" t="n"/>
-      <c r="E82" s="271" t="n">
-        <v>5021000</v>
-      </c>
+      <c r="E82" s="271" t="n"/>
       <c r="F82" s="270" t="n"/>
-      <c r="G82" s="271" t="n">
-        <v>3187000</v>
-      </c>
+      <c r="G82" s="271" t="n"/>
       <c r="H82" s="270" t="n"/>
-      <c r="I82" s="271" t="n">
-        <v>4309000</v>
-      </c>
+      <c r="I82" s="271" t="n"/>
       <c r="J82" s="270" t="n"/>
-      <c r="K82" s="271" t="n">
-        <v>4164000</v>
-      </c>
+      <c r="K82" s="271" t="n"/>
       <c r="L82" s="270" t="n"/>
       <c r="M82" s="13" t="n"/>
       <c r="O82" s="57" t="n">
-        <v>2745000</v>
+        <v>3848000</v>
       </c>
     </row>
     <row r="83" ht="20.1" customHeight="1" s="49">
@@ -4362,25 +4034,17 @@
         </is>
       </c>
       <c r="D83" s="270" t="n"/>
-      <c r="E83" s="271" t="n">
-        <v>4940000</v>
-      </c>
+      <c r="E83" s="271" t="n"/>
       <c r="F83" s="270" t="n"/>
-      <c r="G83" s="271" t="n">
-        <v>5477000</v>
-      </c>
+      <c r="G83" s="271" t="n"/>
       <c r="H83" s="270" t="n"/>
-      <c r="I83" s="271" t="n">
-        <v>5396000</v>
-      </c>
+      <c r="I83" s="271" t="n"/>
       <c r="J83" s="270" t="n"/>
-      <c r="K83" s="271" t="n">
-        <v>4986000</v>
-      </c>
+      <c r="K83" s="271" t="n"/>
       <c r="L83" s="270" t="n"/>
       <c r="M83" s="13" t="n"/>
       <c r="O83" s="57" t="n">
-        <v>5196000</v>
+        <v>4627000</v>
       </c>
     </row>
     <row r="84" ht="20.1" customHeight="1" s="49">
@@ -4391,25 +4055,17 @@
         </is>
       </c>
       <c r="D84" s="270" t="n"/>
-      <c r="E84" s="271" t="n">
-        <v>934000</v>
-      </c>
+      <c r="E84" s="271" t="n"/>
       <c r="F84" s="270" t="n"/>
-      <c r="G84" s="271" t="n">
-        <v>800000</v>
-      </c>
+      <c r="G84" s="271" t="n"/>
       <c r="H84" s="270" t="n"/>
-      <c r="I84" s="271" t="n">
-        <v>1911000</v>
-      </c>
+      <c r="I84" s="271" t="n"/>
       <c r="J84" s="270" t="n"/>
-      <c r="K84" s="271" t="n">
-        <v>2813000</v>
-      </c>
+      <c r="K84" s="271" t="n"/>
       <c r="L84" s="270" t="n"/>
       <c r="M84" s="13" t="n"/>
       <c r="O84" s="57" t="n">
-        <v>1303000</v>
+        <v>2152000</v>
       </c>
     </row>
     <row r="85" ht="20.1" customHeight="1" s="49">
@@ -4420,25 +4076,17 @@
         </is>
       </c>
       <c r="D85" s="270" t="n"/>
-      <c r="E85" s="271" t="n">
-        <v>1046000</v>
-      </c>
+      <c r="E85" s="271" t="n"/>
       <c r="F85" s="270" t="n"/>
-      <c r="G85" s="271" t="n">
-        <v>1175000</v>
-      </c>
+      <c r="G85" s="271" t="n"/>
       <c r="H85" s="270" t="n"/>
-      <c r="I85" s="271" t="n">
-        <v>947000</v>
-      </c>
+      <c r="I85" s="271" t="n"/>
       <c r="J85" s="270" t="n"/>
-      <c r="K85" s="271" t="n">
-        <v>911000</v>
-      </c>
+      <c r="K85" s="271" t="n"/>
       <c r="L85" s="270" t="n"/>
       <c r="M85" s="13" t="n"/>
       <c r="O85" s="58" t="n">
-        <v>912000</v>
+        <v>1106000</v>
       </c>
     </row>
     <row r="86" ht="5.1" customHeight="1" s="49" thickBot="1">
@@ -4813,25 +4461,17 @@
         </is>
       </c>
       <c r="D106" s="283" t="n"/>
-      <c r="E106" s="284" t="n">
-        <v>529000</v>
-      </c>
+      <c r="E106" s="284" t="n"/>
       <c r="F106" s="283" t="n"/>
-      <c r="G106" s="284" t="n">
-        <v>1070000</v>
-      </c>
+      <c r="G106" s="284" t="n"/>
       <c r="H106" s="283" t="n"/>
-      <c r="I106" s="284" t="n">
-        <v>608000</v>
-      </c>
+      <c r="I106" s="284" t="n"/>
       <c r="J106" s="283" t="n"/>
-      <c r="K106" s="285" t="n">
-        <v>759000</v>
-      </c>
+      <c r="K106" s="285" t="n"/>
       <c r="L106" s="286" t="n"/>
       <c r="M106" s="13" t="n"/>
       <c r="O106" s="56" t="n">
-        <v>631000</v>
+        <v>899000</v>
       </c>
     </row>
     <row r="107" ht="27" customHeight="1" s="49">
@@ -4842,25 +4482,17 @@
         </is>
       </c>
       <c r="D107" s="270" t="n"/>
-      <c r="E107" s="288" t="n">
-        <v>1231000</v>
-      </c>
+      <c r="E107" s="288" t="n"/>
       <c r="F107" s="270" t="n"/>
-      <c r="G107" s="288" t="n">
-        <v>796000</v>
-      </c>
+      <c r="G107" s="288" t="n"/>
       <c r="H107" s="270" t="n"/>
-      <c r="I107" s="288" t="n">
-        <v>965000</v>
-      </c>
+      <c r="I107" s="288" t="n"/>
       <c r="J107" s="270" t="n"/>
-      <c r="K107" s="289" t="n">
-        <v>1108000</v>
-      </c>
+      <c r="K107" s="289" t="n"/>
       <c r="L107" s="290" t="n"/>
       <c r="M107" s="13" t="n"/>
       <c r="O107" s="57" t="n">
-        <v>1000000</v>
+        <v>861000</v>
       </c>
     </row>
     <row r="108" ht="27" customHeight="1" s="49" thickBot="1">
@@ -4871,25 +4503,17 @@
         </is>
       </c>
       <c r="D108" s="292" t="n"/>
-      <c r="E108" s="293" t="n">
-        <v>1346000</v>
-      </c>
+      <c r="E108" s="293" t="n"/>
       <c r="F108" s="292" t="n"/>
-      <c r="G108" s="293" t="n">
-        <v>1217000</v>
-      </c>
+      <c r="G108" s="293" t="n"/>
       <c r="H108" s="292" t="n"/>
-      <c r="I108" s="293" t="n">
-        <v>1464000</v>
-      </c>
+      <c r="I108" s="293" t="n"/>
       <c r="J108" s="292" t="n"/>
-      <c r="K108" s="294" t="n">
-        <v>810000</v>
-      </c>
+      <c r="K108" s="294" t="n"/>
       <c r="L108" s="295" t="n"/>
       <c r="M108" s="13" t="n"/>
       <c r="O108" s="58" t="n">
-        <v>1253000</v>
+        <v>669000</v>
       </c>
     </row>
     <row r="109">

</xml_diff>